<commit_message>
Complete practice spreadsheet requirements
</commit_message>
<xml_diff>
--- a/Психологический_центр_готово/04_Практика_3_Excel/Практика3_Электронные_таблицы.xlsx
+++ b/Психологический_центр_готово/04_Практика_3_Excel/Практика3_Электронные_таблицы.xlsx
@@ -13,18 +13,24 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Задание 4" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Задание 5" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Задание 6" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Задание 7" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Задание 8" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Задание 9" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Задание 10" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0 &quot;руб.&quot;"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,12 +39,21 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -51,7 +66,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEDEA"/>
+        <fgColor rgb="00DCEAF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,23 +80,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="009BB7B4"/>
+        <color rgb="008A8F98"/>
       </left>
       <right style="thin">
-        <color rgb="009BB7B4"/>
+        <color rgb="008A8F98"/>
       </right>
       <top style="thin">
-        <color rgb="009BB7B4"/>
+        <color rgb="008A8F98"/>
       </top>
       <bottom style="thin">
-        <color rgb="009BB7B4"/>
+        <color rgb="008A8F98"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -92,6 +107,24 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -100,21 +133,21 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00F4B6B2"/>
+          <fgColor rgb="00F4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00F6E59A"/>
+          <fgColor rgb="00FFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00B8D9C2"/>
+          <fgColor rgb="00D9EAD3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -193,6 +226,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -203,7 +237,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Динамика осадков</a:t>
+              <a:t>Численность студентов из расчета на 1000 человек населения</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -218,7 +252,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Задание 5'!B1</f>
+              <f>'Задание 10'!C1</f>
             </strRef>
           </tx>
           <spPr>
@@ -228,12 +262,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Задание 5'!$A$2:$A$8</f>
+              <f>'Задание 10'!$B$2:$B$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Задание 5'!$B$2:$B$8</f>
+              <f>'Задание 10'!$C$2:$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -242,7 +276,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Задание 5'!C1</f>
+              <f>'Задание 10'!D1</f>
             </strRef>
           </tx>
           <spPr>
@@ -252,12 +286,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Задание 5'!$A$2:$A$8</f>
+              <f>'Задание 10'!$B$2:$B$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Задание 5'!$C$2:$C$8</f>
+              <f>'Задание 10'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -266,7 +300,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Задание 5'!D1</f>
+              <f>'Задание 10'!E1</f>
             </strRef>
           </tx>
           <spPr>
@@ -276,12 +310,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Задание 5'!$A$2:$A$8</f>
+              <f>'Задание 10'!$B$2:$B$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Задание 5'!$D$2:$D$8</f>
+              <f>'Задание 10'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -290,7 +324,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Задание 5'!E1</f>
+              <f>'Задание 10'!F1</f>
             </strRef>
           </tx>
           <spPr>
@@ -300,12 +334,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Задание 5'!$A$2:$A$8</f>
+              <f>'Задание 10'!$B$2:$B$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Задание 5'!$E$2:$E$8</f>
+              <f>'Задание 10'!$F$2:$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -328,7 +362,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Месяц</a:t>
+                  <a:t>Группа</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -355,7 +389,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Размер осадков</a:t>
+                  <a:t>Студентов на 1000 человек</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -384,7 +418,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2700000"/>
+    <ext cx="6480000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -691,12 +725,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="72" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -710,7 +745,6 @@
           <t>Значение</t>
         </is>
       </c>
-      <c r="C1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -721,7 +755,6 @@
       <c r="B2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -732,34 +765,34 @@
       <c r="B3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C3" s="2" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-    </row>
+    </row>
+    <row r="4"/>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Выражение</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Вариант</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Формула Excel</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Результат</t>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Расчет</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Ожидаемый ответ</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>а</t>
         </is>
       </c>
       <c r="B6" s="2">
@@ -770,6 +803,9 @@
         <f>B2^2+(B2+B3)/B3</f>
         <v/>
       </c>
+      <c r="D6" s="2" t="n">
+        <v>10.75</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -785,6 +821,9 @@
         <f>((B2+1)^2)/(2*(B3-1))+((B3+B2)^2)/(2*B3)</f>
         <v/>
       </c>
+      <c r="D7" s="2" t="n">
+        <v>8.791700000000001</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -800,9 +839,157 @@
         <f>(B3-B2+(B2^2+B3)/(B3-B2))/(B2^2+B3^2+(B3*(B2+1))/(4-B2))</f>
         <v/>
       </c>
+      <c r="D8" s="2" t="n">
+        <v>0.3415</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Группа</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Россия</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Китай</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Украина</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -816,7 +1003,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -968,7 +1155,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -981,7 +1169,7 @@
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1107,7 +1295,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -1117,14 +1306,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1145,6 +1335,9 @@
       <c r="E1" s="1" t="n">
         <v>4</v>
       </c>
+      <c r="F1" s="1" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1166,6 +1359,10 @@
         <f>$A2*E$1</f>
         <v/>
       </c>
+      <c r="F2" s="2">
+        <f>$A2*F$1</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1187,6 +1384,10 @@
         <f>$A3*E$1</f>
         <v/>
       </c>
+      <c r="F3" s="2">
+        <f>$A3*F$1</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1208,6 +1409,10 @@
         <f>$A4*E$1</f>
         <v/>
       </c>
+      <c r="F4" s="2">
+        <f>$A4*F$1</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1229,6 +1434,10 @@
         <f>$A5*E$1</f>
         <v/>
       </c>
+      <c r="F5" s="2">
+        <f>$A5*F$1</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1250,9 +1459,14 @@
         <f>$A6*E$1</f>
         <v/>
       </c>
+      <c r="F6" s="2">
+        <f>$A6*F$1</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -1265,12 +1479,12 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1311,19 +1525,19 @@
           <t>Февраль</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="4">
         <f>AVERAGE(B2:E2)</f>
         <v/>
       </c>
@@ -1334,19 +1548,19 @@
           <t>Март</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="D3" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="4">
         <f>AVERAGE(B3:E3)</f>
         <v/>
       </c>
@@ -1357,19 +1571,19 @@
           <t>Апрель</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="4">
         <f>AVERAGE(B4:E4)</f>
         <v/>
       </c>
@@ -1380,19 +1594,19 @@
           <t>Май</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="B5" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D5" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="4">
         <f>AVERAGE(B5:E5)</f>
         <v/>
       </c>
@@ -1403,19 +1617,19 @@
           <t>Июнь</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="C6" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D6" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="4">
         <f>AVERAGE(B6:E6)</f>
         <v/>
       </c>
@@ -1426,19 +1640,19 @@
           <t>Июль</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="C7" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="4">
         <f>AVERAGE(B7:E7)</f>
         <v/>
       </c>
@@ -1449,19 +1663,19 @@
           <t>Август</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="C8" s="2" t="n">
+      <c r="B8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="F8" s="2">
+      <c r="F8" s="4">
         <f>AVERAGE(B8:E8)</f>
         <v/>
       </c>
@@ -1472,23 +1686,23 @@
           <t>Минимальная</t>
         </is>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="4">
         <f>MIN(B2:B8)</f>
         <v/>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="4">
         <f>MIN(C2:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="4">
         <f>MIN(D2:D8)</f>
         <v/>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="4">
         <f>MIN(E2:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="4">
         <f>MIN(F2:F8)</f>
         <v/>
       </c>
@@ -1499,43 +1713,43 @@
           <t>Максимальная</t>
         </is>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="4">
         <f>MAX(B2:B8)</f>
         <v/>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="4">
         <f>MAX(C2:C8)</f>
         <v/>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="4">
         <f>MAX(D2:D8)</f>
         <v/>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="4">
         <f>MAX(E2:E8)</f>
         <v/>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="4">
         <f>MAX(F2:F8)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:F10">
+  <conditionalFormatting sqref="B2:E8">
     <cfRule type="cellIs" priority="1" operator="between" dxfId="0">
       <formula>0</formula>
       <formula>12</formula>
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
-      <formula>13</formula>
+      <formula>12.0001</formula>
       <formula>18</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>18</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -1549,232 +1763,968 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Время</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Аудитория</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Группы</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Суббота, 22.05.2021</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>09.00:10.30</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>520</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Ув-741, Мв-741</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Суббота, 22.05.2021</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>10.40:12.10</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr"/>
+      <c r="D3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Суббота, 22.05.2021</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>12.40:14.10</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>520</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Эв-741</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Суббота, 22.05.2021</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>14.20:15.50</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Пятница, 28.05.2021</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>17.40:19.10</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Мв-721, Жв-721, Эв-721</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Пятница, 28.05.2021</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>19.20:20.50</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Суббота, 29.05.2021</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>09.00:10.30</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>ВУв-641, ВЭв-641</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Суббота, 29.05.2021</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>10.40:12.10</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr"/>
+      <c r="D9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Понедельник, 31.05.2021</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>17.40</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Мв-721, Жв-721, Эв-721</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Фамилия</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Лежа</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>С колена</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Стоя</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Сумма</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Отобран</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Иванов И.И.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F2" s="2">
+        <f>SUM(C2:E2)</f>
+        <v/>
+      </c>
+      <c r="G2" s="2">
+        <f>IF(F2&gt;=290,"Да","Нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Петров П.П.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="F3" s="2">
+        <f>SUM(C3:E3)</f>
+        <v/>
+      </c>
+      <c r="G3" s="2">
+        <f>IF(F3&gt;=290,"Да","Нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Сидоров С.С.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="F4" s="2">
+        <f>SUM(C4:E4)</f>
+        <v/>
+      </c>
+      <c r="G4" s="2">
+        <f>IF(F4&gt;=290,"Да","Нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Кузнецов А.А.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F5" s="2">
+        <f>SUM(C5:E5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="2">
+        <f>IF(F5&gt;=290,"Да","Нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Смирнов Д.Д.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="F6" s="2">
+        <f>SUM(C6:E6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="2">
+        <f>IF(F6&gt;=290,"Да","Нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Орлов Р.Р.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="F7" s="2">
+        <f>SUM(C7:E7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="2">
+        <f>IF(F7&gt;=290,"Да","Нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Васильев М.М.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F8" s="2">
+        <f>SUM(C8:E8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="2">
+        <f>IF(F8&gt;=290,"Да","Нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Морозов Н.Н.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="F9" s="2">
+        <f>SUM(C9:E9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="2">
+        <f>IF(F9&gt;=290,"Да","Нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Федоров К.К.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F10" s="2">
+        <f>SUM(C10:E10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="2">
+        <f>IF(F10&gt;=290,"Да","Нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Егоров Е.Е.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F11" s="2">
+        <f>SUM(C11:E11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="2">
+        <f>IF(F11&gt;=290,"Да","Нет")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Дата</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Время</t>
+          <t>ФИО</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Количество продаж</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Аудитория</t>
+          <t>Размер изменения оплаты труда</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Группа</t>
+          <t>Размер оплаты труда за месяц</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Суббота, 22.05.2021</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>09.00:10.30</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>420</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Ув-741</t>
-        </is>
+          <t>Иванов И.И.</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="C2" s="9">
+        <f>IF(B2&gt;20,(B2-20)*50,IF(B2&lt;20,-(20-B2)*100,0))</f>
+        <v/>
+      </c>
+      <c r="D2" s="9">
+        <f>2000+C2</f>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Суббота, 22.05.2021</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>10.40:12.10</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>520</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Мв-741</t>
-        </is>
+          <t>Петров П.П.</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="C3" s="9">
+        <f>IF(B3&gt;20,(B3-20)*50,IF(B3&lt;20,-(20-B3)*100,0))</f>
+        <v/>
+      </c>
+      <c r="D3" s="9">
+        <f>2000+C3</f>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Суббота, 22.05.2021</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>12.40:14.10</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>520</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Эв-741</t>
-        </is>
+          <t>Сидоров С.С.</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" s="9">
+        <f>IF(B4&gt;20,(B4-20)*50,IF(B4&lt;20,-(20-B4)*100,0))</f>
+        <v/>
+      </c>
+      <c r="D4" s="9">
+        <f>2000+C4</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Пятница, 28.05.2021</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>14.20:15.50</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>420</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Мв-721</t>
-        </is>
+          <t>Кузнецова А.А.</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="C5" s="9">
+        <f>IF(B5&gt;20,(B5-20)*50,IF(B5&lt;20,-(20-B5)*100,0))</f>
+        <v/>
+      </c>
+      <c r="D5" s="9">
+        <f>2000+C5</f>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Пятница, 28.05.2021</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>17.40:19.10</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>420</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Жв-721</t>
-        </is>
+          <t>Смирнова Е.Е.</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" s="9">
+        <f>IF(B6&gt;20,(B6-20)*50,IF(B6&lt;20,-(20-B6)*100,0))</f>
+        <v/>
+      </c>
+      <c r="D6" s="9">
+        <f>2000+C6</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Пятница, 28.05.2021</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>19.20:20.50</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>420</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Эв-721</t>
-        </is>
+          <t>Орлова М.М.</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="C7" s="9">
+        <f>IF(B7&gt;20,(B7-20)*50,IF(B7&lt;20,-(20-B7)*100,0))</f>
+        <v/>
+      </c>
+      <c r="D7" s="9">
+        <f>2000+C7</f>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Суббота, 29.05.2021</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>09.00:10.30</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>520</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>ВУв-641</t>
-        </is>
+          <t>Морозов Н.Н.</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="C8" s="9">
+        <f>IF(B8&gt;20,(B8-20)*50,IF(B8&lt;20,-(20-B8)*100,0))</f>
+        <v/>
+      </c>
+      <c r="D8" s="9">
+        <f>2000+C8</f>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Суббота, 29.05.2021</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>10.40:12.10</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>520</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>ВЭв-641</t>
-        </is>
+          <t>Федоров К.К.</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="C9" s="9">
+        <f>IF(B9&gt;20,(B9-20)*50,IF(B9&lt;20,-(20-B9)*100,0))</f>
+        <v/>
+      </c>
+      <c r="D9" s="9">
+        <f>2000+C9</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Понедельник, 31.05.2021</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>17.40</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>420</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Мв-721, Жв-721, Эв-721</t>
-        </is>
+          <t>Егоров Р.Р.</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="C10" s="9">
+        <f>IF(B10&gt;20,(B10-20)*50,IF(B10&lt;20,-(20-B10)*100,0))</f>
+        <v/>
+      </c>
+      <c r="D10" s="9">
+        <f>2000+C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Васильев Д.Д.</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="C11" s="9">
+        <f>IF(B11&gt;20,(B11-20)*50,IF(B11&lt;20,-(20-B11)*100,0))</f>
+        <v/>
+      </c>
+      <c r="D11" s="9">
+        <f>2000+C11</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Ф.И.О.</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Решение</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Иванов И.И.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>172</v>
+      </c>
+      <c r="D2" s="2">
+        <f>IF(AND(C2&gt;=168,C2&lt;=178),"принят","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Петрова Л.П.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="D3" s="2">
+        <f>IF(AND(C3&gt;=168,C3&lt;=178),"принят","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Сидорова А.А.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="D4" s="2">
+        <f>IF(AND(C4&gt;=168,C4&lt;=178),"принят","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Кузнецов Р.Р.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>178</v>
+      </c>
+      <c r="D5" s="2">
+        <f>IF(AND(C5&gt;=168,C5&lt;=178),"принят","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Смирнова Е.Е.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>165</v>
+      </c>
+      <c r="D6" s="2">
+        <f>IF(AND(C6&gt;=168,C6&lt;=178),"принят","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Орлов М.М.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>174</v>
+      </c>
+      <c r="D7" s="2">
+        <f>IF(AND(C7&gt;=168,C7&lt;=178),"принят","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Морозова Н.Н.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>181</v>
+      </c>
+      <c r="D8" s="2">
+        <f>IF(AND(C8&gt;=168,C8&lt;=178),"принят","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Федорова К.К.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="D9" s="2">
+        <f>IF(AND(C9&gt;=168,C9&lt;=178),"принят","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Васильев Д.Д.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="D10" s="2">
+        <f>IF(AND(C10&gt;=168,C10&lt;=178),"принят","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Егорова Е.Ф.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>167</v>
+      </c>
+      <c r="D11" s="2">
+        <f>IF(AND(C11&gt;=168,C11&lt;=178),"принят","нет")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>